<commit_message>
Update class stats, ability balance, and friendly equipment
</commit_message>
<xml_diff>
--- a/CLASS_ABILITIES.xlsx
+++ b/CLASS_ABILITIES.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archer" sheetId="1" r:id="R1ab8ac45c29b4288"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleric" sheetId="2" r:id="R88a8eb222de94449"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warrior" sheetId="3" r:id="Rc6e88f29e3464958"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wizard" sheetId="4" r:id="Rd58e949af40e4fc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archer" sheetId="1" r:id="R8ddaf0e317fa4e43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleric" sheetId="2" r:id="R558d3e0230d84f72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warrior" sheetId="3" r:id="R1b56a7eb5df943dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wizard" sheetId="4" r:id="R58e2d3f33e294eba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -567,7 +567,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R061cfa2b1f084a94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7709501438a9456b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -764,7 +764,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffde7ddaff8e4e80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0226d02a7fbf4d46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1012,7 +1012,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R683313d513504dba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R765c52455b044463"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1132,7 +1132,7 @@
         <x:v>Fireball</x:v>
       </x:c>
       <x:c r="E8" s="19" t="str">
-        <x:v>Magic ability. Projectile. Range 8.00. Magical damage (10 innate + Intelligence x100%). Affects: enemies. Can aim at a cell. Area: circle, 7-cell span. No weapon required.</x:v>
+        <x:v>Magic ability. Projectile. Range 8.00. Magical damage (5 innate + Intelligence x100%). Affects: enemies. Can aim at a cell. Area: circle, 5-cell span. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -1209,7 +1209,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R807aeb955da64db6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4406395fd39742f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>